<commit_message>
Recreate Excel file with formatting and add CSV version for easier access
</commit_message>
<xml_diff>
--- a/outputs/reports/dcca_newtown_intersection.xlsx
+++ b/outputs/reports/dcca_newtown_intersection.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +28,23 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00366092"/>
+        <bgColor rgb="00366092"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -57,7 +67,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
Add Ma On Shan as separate New Town with its DCCAs (11 in 2001, 12 in 2006)
</commit_message>
<xml_diff>
--- a/outputs/reports/dcca_newtown_intersection.xlsx
+++ b/outputs/reports/dcca_newtown_intersection.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C317"/>
+  <dimension ref="A1:C340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -931,7 +931,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -946,12 +946,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Sha Tin - Chui Tin</t>
+          <t>Sha Tin - Heng On</t>
         </is>
       </c>
     </row>
@@ -961,12 +961,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Sha Tin - Chun Kam</t>
+          <t>Sha Tin - Heng To</t>
         </is>
       </c>
     </row>
@@ -976,12 +976,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Sha Tin - Chun Ma</t>
+          <t>Sha Tin - Kam Fung</t>
         </is>
       </c>
     </row>
@@ -991,12 +991,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sha Tin - City One</t>
+          <t>Sha Tin - Kam Ying</t>
         </is>
       </c>
     </row>
@@ -1006,12 +1006,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Sha Tin - Fo Tan</t>
+          <t>Sha Tin - Lee On</t>
         </is>
       </c>
     </row>
@@ -1021,12 +1021,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Sha Tin - Heng To</t>
+          <t>Sha Tin - Saddle Ridge</t>
         </is>
       </c>
     </row>
@@ -1036,12 +1036,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Sha Tin - Hin Ka</t>
+          <t>Sha Tin - Sunshine City</t>
         </is>
       </c>
     </row>
@@ -1051,12 +1051,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Sha Tin - Jat Min</t>
+          <t>Sha Tin - Tai Shui Hang</t>
         </is>
       </c>
     </row>
@@ -1066,12 +1066,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Sha Tin - Keng Hau</t>
+          <t>Sha Tin - Yiu On</t>
         </is>
       </c>
     </row>
@@ -1081,12 +1081,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Sha Tin - Kwong Hong</t>
+          <t>Tai Po - Sai Kung North</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sha Tin - Kwong Yuen</t>
+          <t>Sha Tin - Bik Woo</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Sha Tin - Lek Yuen</t>
+          <t>Sha Tin - Chui Tin</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Sha Tin - Lower Shing Mun</t>
+          <t>Sha Tin - Chun Kam</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Sha Tin - May Shing</t>
+          <t>Sha Tin - Chun Ma</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Sha Tin - Mei Tin</t>
+          <t>Sha Tin - City One</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Sha Tin - Pok Hong</t>
+          <t>Sha Tin - Fo Tan</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Sha Tin - Sha Kok</t>
+          <t>Sha Tin - Heng To</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Sha Tin - Sha Tin Town Centre</t>
+          <t>Sha Tin - Hin Ka</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Sha Tin - Sui Wo</t>
+          <t>Sha Tin - Jat Min</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Sha Tin - Sun Chui</t>
+          <t>Sha Tin - Keng Hau</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Sha Tin - Sun Tin Wai</t>
+          <t>Sha Tin - Kwong Hong</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Sha Tin - Tai Shui Hang</t>
+          <t>Sha Tin - Kwong Yuen</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sha Tin - Tai Wai</t>
+          <t>Sha Tin - Lek Yuen</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Sha Tin - Tin Sum</t>
+          <t>Sha Tin - Lower Shing Mun</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sha Tin - Tsang Tai Uk</t>
+          <t>Sha Tin - May Shing</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Sha Tin - Wo Che Estate</t>
+          <t>Sha Tin - Mei Tin</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Sha Tin - Wong Uk</t>
+          <t>Sha Tin - Pok Hong</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Sha Tin - Yue Shing</t>
+          <t>Sha Tin - Sha Kok</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Tai Po - Tai Po Kau</t>
+          <t>Sha Tin - Sha Tin Town Centre</t>
         </is>
       </c>
     </row>
@@ -1381,12 +1381,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Yuen Long - Ha Tsuen</t>
+          <t>Sha Tin - Sui Wo</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Yuen Long - Kingswood North</t>
+          <t>Sha Tin - Sun Chui</t>
         </is>
       </c>
     </row>
@@ -1411,12 +1411,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Yuen Long - Kingswood South</t>
+          <t>Sha Tin - Sun Tin Wai</t>
         </is>
       </c>
     </row>
@@ -1426,12 +1426,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Yuen Long - Ping Shan North</t>
+          <t>Sha Tin - Tai Shui Hang</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Yuen Long - Shui Oi</t>
+          <t>Sha Tin - Tai Wai</t>
         </is>
       </c>
     </row>
@@ -1456,12 +1456,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Yuen Long - Tin Shui</t>
+          <t>Sha Tin - Tin Sum</t>
         </is>
       </c>
     </row>
@@ -1471,12 +1471,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Yuen Long - Tin Tsz</t>
+          <t>Sha Tin - Tsang Tai Uk</t>
         </is>
       </c>
     </row>
@@ -1486,12 +1486,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Yuen Long - Tin Yiu</t>
+          <t>Sha Tin - Wo Che Estate</t>
         </is>
       </c>
     </row>
@@ -1501,12 +1501,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Yuen Long - Yiu Yau</t>
+          <t>Sha Tin - Wong Uk</t>
         </is>
       </c>
     </row>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Kwun Tong - Kwong Tak</t>
+          <t>Sha Tin - Yue Shing</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Kwun Tong - Tak Tin</t>
+          <t>Tai Po - Tai Po Kau</t>
         </is>
       </c>
     </row>
@@ -1546,12 +1546,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Kwun Tong - Yau Tong Sze Shan</t>
+          <t>Yuen Long - Ha Tsuen</t>
         </is>
       </c>
     </row>
@@ -1561,12 +1561,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Sai Kung - Fu Yu</t>
+          <t>Yuen Long - Kingswood North</t>
         </is>
       </c>
     </row>
@@ -1576,12 +1576,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Sai Kung - Hang Hau East</t>
+          <t>Yuen Long - Kingswood South</t>
         </is>
       </c>
     </row>
@@ -1591,12 +1591,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Sai Kung - Hang Hau West</t>
+          <t>Yuen Long - Ping Shan North</t>
         </is>
       </c>
     </row>
@@ -1606,12 +1606,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Sai Kung - Hau Tak</t>
+          <t>Yuen Long - Shui Oi</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1621,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Sai Kung - Hong King</t>
+          <t>Yuen Long - Tin Shui</t>
         </is>
       </c>
     </row>
@@ -1636,12 +1636,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Sai Kung - King Lam</t>
+          <t>Yuen Long - Tin Tsz</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Sai Kung - Kwong Ming</t>
+          <t>Yuen Long - Tin Yiu</t>
         </is>
       </c>
     </row>
@@ -1666,12 +1666,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Sai Kung - On Hong</t>
+          <t>Yuen Long - Yiu Yau</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Sai Kung - Po Lam</t>
+          <t>Kwun Tong - Kwong Tak</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Sai Kung - Sheung Tak</t>
+          <t>Kwun Tong - Tak Tin</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Sai Kung - Tsui Lam</t>
+          <t>Kwun Tong - Yau Tong Sze Shan</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Sai Kung - Tung Ming</t>
+          <t>Sai Kung - Fu Yu</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Sai Kung - Wan Hang</t>
+          <t>Sai Kung - Hang Hau East</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Sai Kung - Yan Ying</t>
+          <t>Sai Kung - Hang Hau West</t>
         </is>
       </c>
     </row>
@@ -1771,12 +1771,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Chung Estate</t>
+          <t>Sai Kung - Hau Tak</t>
         </is>
       </c>
     </row>
@@ -1786,12 +1786,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Shing West Estate</t>
+          <t>Sai Kung - Hong King</t>
         </is>
       </c>
     </row>
@@ -1801,12 +1801,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Lower Tai Wo Hau</t>
+          <t>Sai Kung - King Lam</t>
         </is>
       </c>
     </row>
@@ -1816,12 +1816,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Shek Yam</t>
+          <t>Sai Kung - Kwong Ming</t>
         </is>
       </c>
     </row>
@@ -1831,12 +1831,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Allway</t>
+          <t>Sai Kung - On Hong</t>
         </is>
       </c>
     </row>
@@ -1846,12 +1846,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Cheung Shan</t>
+          <t>Sai Kung - Po Lam</t>
         </is>
       </c>
     </row>
@@ -1861,12 +1861,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Clague Garden</t>
+          <t>Sai Kung - Sheung Tak</t>
         </is>
       </c>
     </row>
@@ -1876,12 +1876,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Discovery Park</t>
+          <t>Sai Kung - Tsui Lam</t>
         </is>
       </c>
     </row>
@@ -1891,12 +1891,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Fuk Loi</t>
+          <t>Sai Kung - Tung Ming</t>
         </is>
       </c>
     </row>
@@ -1906,12 +1906,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Hoi Bun</t>
+          <t>Sai Kung - Wan Hang</t>
         </is>
       </c>
     </row>
@@ -1921,12 +1921,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lai Hing</t>
+          <t>Sai Kung - Yan Ying</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lai To</t>
+          <t>Kwai Tsing - Kwai Chung Estate</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lei Muk Shue East</t>
+          <t>Kwai Tsing - Kwai Shing West Estate</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lei Muk Shue West</t>
+          <t>Kwai Tsing - Lower Tai Wo Hau</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Luk Yeung</t>
+          <t>Kwai Tsing - Shek Yam</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Shek Wai Kok</t>
+          <t>Tsuen Wan - Allway</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tak Wah</t>
+          <t>Tsuen Wan - Cheung Shan</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tsuen Wan Centre</t>
+          <t>Tsuen Wan - Clague Garden</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tsuen Wan Rural East</t>
+          <t>Tsuen Wan - Discovery Park</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tsuen Wan Rural West</t>
+          <t>Tsuen Wan - Fuk Loi</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Yeung Uk Road</t>
+          <t>Tsuen Wan - Hoi Bun</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Tuen Mun - Sam Shing</t>
+          <t>Tsuen Wan - Lai Hing</t>
         </is>
       </c>
     </row>
@@ -2101,12 +2101,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tsuen Wan Rural West</t>
+          <t>Tsuen Wan - Lai To</t>
         </is>
       </c>
     </row>
@@ -2116,12 +2116,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Tuen Mun - Butterfly</t>
+          <t>Tsuen Wan - Lei Muk Shue East</t>
         </is>
       </c>
     </row>
@@ -2131,12 +2131,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Tuen Mun - Handsome</t>
+          <t>Tsuen Wan - Lei Muk Shue West</t>
         </is>
       </c>
     </row>
@@ -2146,12 +2146,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Tuen Mun - Hing Tsak</t>
+          <t>Tsuen Wan - Luk Yeung</t>
         </is>
       </c>
     </row>
@@ -2161,12 +2161,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Tuen Mun - Kin Sang</t>
+          <t>Tsuen Wan - Shek Wai Kok</t>
         </is>
       </c>
     </row>
@@ -2176,12 +2176,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Tuen Mun - Leung King</t>
+          <t>Tsuen Wan - Tak Wah</t>
         </is>
       </c>
     </row>
@@ -2191,12 +2191,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Tuen Mun - Lok Tsui</t>
+          <t>Tsuen Wan - Tsuen Wan Centre</t>
         </is>
       </c>
     </row>
@@ -2206,12 +2206,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Tuen Mun - Lung Mun</t>
+          <t>Tsuen Wan - Tsuen Wan Rural East</t>
         </is>
       </c>
     </row>
@@ -2221,12 +2221,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Tuen Mun - On Ting</t>
+          <t>Tsuen Wan - Tsuen Wan Rural West</t>
         </is>
       </c>
     </row>
@@ -2236,12 +2236,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Tuen Mun - Prime View</t>
+          <t>Tsuen Wan - Yeung Uk Road</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Tuen Mun - San Hui</t>
+          <t>Tsuen Wan - Tsuen Wan Rural West</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Tuen Mun - San King</t>
+          <t>Tuen Mun - Butterfly</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Tuen Mun - Shan King North</t>
+          <t>Tuen Mun - Handsome</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Tuen Mun - Shan King South</t>
+          <t>Tuen Mun - Hing Tsak</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Chi</t>
+          <t>Tuen Mun - Kin Sang</t>
         </is>
       </c>
     </row>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Hei</t>
+          <t>Tuen Mun - Leung King</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Hong</t>
+          <t>Tuen Mun - Lok Tsui</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Lun</t>
+          <t>Tuen Mun - Lung Mun</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Sun</t>
+          <t>Tuen Mun - On Ting</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2406,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tai Hing South</t>
+          <t>Tuen Mun - Prime View</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tin King</t>
+          <t>Tuen Mun - Sam Shing</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tsui Fook</t>
+          <t>Tuen Mun - San Hui</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tsui Hing</t>
+          <t>Tuen Mun - San King</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tuen Mun Rural</t>
+          <t>Tuen Mun - Shan King North</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tuen Mun Town Centre</t>
+          <t>Tuen Mun - Shan King South</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Tuen Mun - Wu King</t>
+          <t>Tuen Mun - Siu Chi</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Tuen Mun - Yau Oi North</t>
+          <t>Tuen Mun - Siu Hei</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Tuen Mun - Yau Oi South</t>
+          <t>Tuen Mun - Siu Hong</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Tuen Mun - Yuet Wu</t>
+          <t>Tuen Mun - Siu Lun</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Yuen Long - Ha Tsuen</t>
+          <t>Tuen Mun - Siu Sun</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Yuen Long - Ping Shan South</t>
+          <t>Tuen Mun - Tai Hing South</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Yuen Long - Shap Pat Heung South</t>
+          <t>Tuen Mun - Tin King</t>
         </is>
       </c>
     </row>
@@ -2596,12 +2596,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Yuen Long - Fung Cheung</t>
+          <t>Tuen Mun - Tsui Fook</t>
         </is>
       </c>
     </row>
@@ -2611,12 +2611,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Yuen Long - Fung Nin</t>
+          <t>Tuen Mun - Tsui Hing</t>
         </is>
       </c>
     </row>
@@ -2626,12 +2626,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Yuen Long - Nam Ping</t>
+          <t>Tuen Mun - Tuen Mun Rural</t>
         </is>
       </c>
     </row>
@@ -2641,12 +2641,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Yuen Long - Pek Long</t>
+          <t>Tuen Mun - Tuen Mun Town Centre</t>
         </is>
       </c>
     </row>
@@ -2656,12 +2656,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Yuen Long - Ping Shan North</t>
+          <t>Tuen Mun - Wu King</t>
         </is>
       </c>
     </row>
@@ -2671,12 +2671,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Yuen Long - Ping Shan South</t>
+          <t>Tuen Mun - Yau Oi North</t>
         </is>
       </c>
     </row>
@@ -2686,12 +2686,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Yuen Long - San Tin</t>
+          <t>Tuen Mun - Yau Oi South</t>
         </is>
       </c>
     </row>
@@ -2701,12 +2701,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Yuen Long - Shap Pat Heung North</t>
+          <t>Tuen Mun - Yuet Wu</t>
         </is>
       </c>
     </row>
@@ -2716,12 +2716,12 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Yuen Long - Shap Pat Heung South</t>
+          <t>Yuen Long - Ha Tsuen</t>
         </is>
       </c>
     </row>
@@ -2731,12 +2731,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Yuen Long - Shui Pin</t>
+          <t>Yuen Long - Ping Shan South</t>
         </is>
       </c>
     </row>
@@ -2746,177 +2746,177 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Yuen Long - Tai Kiu</t>
+          <t>Yuen Long - Shap Pat Heung South</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Cho Yiu</t>
+          <t>Yuen Long - Fung Cheung</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Hing Fong</t>
+          <t>Yuen Long - Fung Nin</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Chung Estate</t>
+          <t>Yuen Long - Nam Ping</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Fong</t>
+          <t>Yuen Long - Pek Long</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Hing</t>
+          <t>Yuen Long - Ping Shan North</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Shing East Estate</t>
+          <t>Yuen Long - Ping Shan South</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Shing West Estate</t>
+          <t>Yuen Long - San Tin</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Lai King</t>
+          <t>Yuen Long - Shap Pat Heung North</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Lai Wah</t>
+          <t>Yuen Long - Shap Pat Heung South</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Lai Yiu</t>
+          <t>Yuen Long - Shui Pin</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Kwai Chung</t>
+          <t>Yuen Long</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Lower Tai Wo Hau</t>
+          <t>Yuen Long - Tai Kiu</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Kwai Tsing - On Yam</t>
+          <t>Kwai Tsing - Cho Yiu</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Shek Lei</t>
+          <t>Kwai Tsing - Hing Fong</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Shek Lei Extension</t>
+          <t>Kwai Tsing - Kwai Chung Estate</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Shek Yam</t>
+          <t>Kwai Tsing - Kwai Fong</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Tai Pak Tin</t>
+          <t>Kwai Tsing - Kwai Hing</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3006,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Tsing Yi South</t>
+          <t>Kwai Tsing - Kwai Shing East Estate</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Upper Tai Wo Hau</t>
+          <t>Kwai Tsing - Kwai Shing West Estate</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Sha Tin - Chung Shing</t>
+          <t>Kwai Tsing - Lai King</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Sha Tin - Mei Tin</t>
+          <t>Kwai Tsing - Lai Wah</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Sham Shui Po - Lai Chi Kok</t>
+          <t>Kwai Tsing - Lai Yiu</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Sham Shui Po - Lung Ping</t>
+          <t>Kwai Tsing - Lower Tai Wo Hau</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Sham Shui Po - Mei Foo Central</t>
+          <t>Kwai Tsing - On Yam</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Sham Shui Po - Mei Foo North</t>
+          <t>Kwai Tsing - Shek Lei</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Sham Shui Po - Mei Foo South</t>
+          <t>Kwai Tsing - Shek Lei Extension</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Hoi Bun</t>
+          <t>Kwai Tsing - Shek Yam</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lei Muk Shue East</t>
+          <t>Kwai Tsing - Tai Pak Tin</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lei Muk Shue West</t>
+          <t>Kwai Tsing - Tsing Yi South</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Luk Yeung</t>
+          <t>Kwai Tsing - Upper Tai Wo Hau</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Shek Wai Kok</t>
+          <t>Sha Tin - Chung Shing</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3216,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Yeung Uk Road</t>
+          <t>Sha Tin - Mei Tin</t>
         </is>
       </c>
     </row>
@@ -3226,12 +3226,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Sha Tin - Bik Woo</t>
+          <t>Sham Shui Po - Lai Chi Kok</t>
         </is>
       </c>
     </row>
@@ -3241,12 +3241,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Sha Tin - Chui Tin</t>
+          <t>Sham Shui Po - Lung Ping</t>
         </is>
       </c>
     </row>
@@ -3256,12 +3256,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Sha Tin - Chun Fung</t>
+          <t>Sham Shui Po - Mei Foo Central</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Sha Tin - Chun Ma</t>
+          <t>Sham Shui Po - Mei Foo North</t>
         </is>
       </c>
     </row>
@@ -3286,12 +3286,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Sha Tin - Chung Shing</t>
+          <t>Sham Shui Po - Mei Foo South</t>
         </is>
       </c>
     </row>
@@ -3301,12 +3301,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Sha Tin - City One</t>
+          <t>Tsuen Wan - Hoi Bun</t>
         </is>
       </c>
     </row>
@@ -3316,12 +3316,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Sha Tin - Fo Tan</t>
+          <t>Tsuen Wan - Lei Muk Shue East</t>
         </is>
       </c>
     </row>
@@ -3331,12 +3331,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Sha Tin - Hin Ka</t>
+          <t>Tsuen Wan - Lei Muk Shue West</t>
         </is>
       </c>
     </row>
@@ -3346,12 +3346,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Sha Tin - Jat Min</t>
+          <t>Tsuen Wan - Luk Yeung</t>
         </is>
       </c>
     </row>
@@ -3361,12 +3361,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Sha Tin - Keng Hau</t>
+          <t>Tsuen Wan - Shek Wai Kok</t>
         </is>
       </c>
     </row>
@@ -3376,12 +3376,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Kwai Chung</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Sha Tin - Kwong Hong</t>
+          <t>Tsuen Wan - Yeung Uk Road</t>
         </is>
       </c>
     </row>
@@ -3391,12 +3391,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Sha Tin - Kwong Yuen</t>
+          <t>Sha Tin - Chung On</t>
         </is>
       </c>
     </row>
@@ -3406,12 +3406,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Sha Tin - Lek Yuen</t>
+          <t>Sha Tin - Fu Lung</t>
         </is>
       </c>
     </row>
@@ -3421,12 +3421,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Sha Tin - Mei Tin</t>
+          <t>Sha Tin - Heng On</t>
         </is>
       </c>
     </row>
@@ -3436,12 +3436,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Sha Tin - On Tai</t>
+          <t>Sha Tin - Kam To</t>
         </is>
       </c>
     </row>
@@ -3451,12 +3451,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Sha Tin - Pok Hong</t>
+          <t>Sha Tin - Kam Ying</t>
         </is>
       </c>
     </row>
@@ -3466,12 +3466,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Sha Tin - Sha Kok</t>
+          <t>Sha Tin - Lee On</t>
         </is>
       </c>
     </row>
@@ -3481,12 +3481,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Sha Tin - Sha Tin Town Centre</t>
+          <t>Sha Tin - On Tai</t>
         </is>
       </c>
     </row>
@@ -3496,12 +3496,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Sha Tin - Sui Wo</t>
+          <t>Sha Tin - Sunshine City</t>
         </is>
       </c>
     </row>
@@ -3511,12 +3511,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Sha Tin - Sun Chui</t>
+          <t>Sha Tin - Tai Shui Hang</t>
         </is>
       </c>
     </row>
@@ -3526,12 +3526,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Sha Tin - Sun Tin Wai</t>
+          <t>Sha Tin - Yiu On</t>
         </is>
       </c>
     </row>
@@ -3541,12 +3541,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Sha Tin - Tai Shui Hang</t>
+          <t>Sha Tin - Yu Yan</t>
         </is>
       </c>
     </row>
@@ -3556,12 +3556,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
+          <t>Ma On Shan</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Sha Tin - Tai Wai</t>
+          <t>Tai Po - Sai Kung North</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Sha Tin - Tin Sum</t>
+          <t>Sha Tin - Bik Woo</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Sha Tin - Wo Che Estate</t>
+          <t>Sha Tin - Chui Tin</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Sha Tin - Wong Uk</t>
+          <t>Sha Tin - Chun Fung</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Sha Tin - Yu Yan</t>
+          <t>Sha Tin - Chun Ma</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Sha Tin - Yue Shing</t>
+          <t>Sha Tin - Chung Shing</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Tai Po - Tai Po Kau</t>
+          <t>Sha Tin - City One</t>
         </is>
       </c>
     </row>
@@ -3661,12 +3661,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Yuen Long - Chung Wah</t>
+          <t>Sha Tin - Fo Tan</t>
         </is>
       </c>
     </row>
@@ -3676,12 +3676,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Yuen Long - Fu Yan</t>
+          <t>Sha Tin - Hin Ka</t>
         </is>
       </c>
     </row>
@@ -3691,12 +3691,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Yuen Long - Ha Tsuen</t>
+          <t>Sha Tin - Jat Min</t>
         </is>
       </c>
     </row>
@@ -3706,12 +3706,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Yuen Long - Kingswood North</t>
+          <t>Sha Tin - Keng Hau</t>
         </is>
       </c>
     </row>
@@ -3721,12 +3721,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Yuen Long - Kingswood South</t>
+          <t>Sha Tin - Kwong Hong</t>
         </is>
       </c>
     </row>
@@ -3736,12 +3736,12 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Yuen Long - Ping Shan North</t>
+          <t>Sha Tin - Kwong Yuen</t>
         </is>
       </c>
     </row>
@@ -3751,12 +3751,12 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Yuen Long - Shui Oi</t>
+          <t>Sha Tin - Lek Yuen</t>
         </is>
       </c>
     </row>
@@ -3766,12 +3766,12 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Yuen Long - Shui Wah</t>
+          <t>Sha Tin - Mei Tin</t>
         </is>
       </c>
     </row>
@@ -3781,12 +3781,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Yuen Long - Tin Heng</t>
+          <t>Sha Tin - On Tai</t>
         </is>
       </c>
     </row>
@@ -3796,12 +3796,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Yuen Long - Tin Shing</t>
+          <t>Sha Tin - Pok Hong</t>
         </is>
       </c>
     </row>
@@ -3811,12 +3811,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Yuen Long - Tin Yiu</t>
+          <t>Sha Tin - Sha Kok</t>
         </is>
       </c>
     </row>
@@ -3826,12 +3826,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Yuen Long - Tsz Yau</t>
+          <t>Sha Tin - Sha Tin Town Centre</t>
         </is>
       </c>
     </row>
@@ -3841,12 +3841,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Yuen Long - Wang Yat</t>
+          <t>Sha Tin - Sui Wo</t>
         </is>
       </c>
     </row>
@@ -3856,12 +3856,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Yuen Long - Yat Chak</t>
+          <t>Sha Tin - Sun Chui</t>
         </is>
       </c>
     </row>
@@ -3871,12 +3871,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Tin Shui Wai</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Yuen Long - Yuet Yan</t>
+          <t>Sha Tin - Sun Tin Wai</t>
         </is>
       </c>
     </row>
@@ -3886,12 +3886,12 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Kwun Tong - Kwong Tak</t>
+          <t>Sha Tin - Tai Shui Hang</t>
         </is>
       </c>
     </row>
@@ -3901,12 +3901,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Kwun Tong - Tak Tin</t>
+          <t>Sha Tin - Tai Wai</t>
         </is>
       </c>
     </row>
@@ -3916,12 +3916,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Kwun Tong - Yau Tong Sze Shan East</t>
+          <t>Sha Tin - Tin Sum</t>
         </is>
       </c>
     </row>
@@ -3931,12 +3931,12 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Kwun Tong - Yau Tong Sze Shan West</t>
+          <t>Sha Tin - Wo Che Estate</t>
         </is>
       </c>
     </row>
@@ -3946,12 +3946,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Sai Kung - Fu Yu</t>
+          <t>Sha Tin - Wong Uk</t>
         </is>
       </c>
     </row>
@@ -3961,12 +3961,12 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Sai Kung - Hang Hau East</t>
+          <t>Sha Tin - Yu Yan</t>
         </is>
       </c>
     </row>
@@ -3976,12 +3976,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Sai Kung - Hang Hau West</t>
+          <t>Sha Tin - Yue Shing</t>
         </is>
       </c>
     </row>
@@ -3991,12 +3991,12 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Sai Kung - Hau Tak</t>
+          <t>Tai Po - Tai Po Kau</t>
         </is>
       </c>
     </row>
@@ -4006,12 +4006,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Sai Kung - Hong King</t>
+          <t>Yuen Long - Chung Wah</t>
         </is>
       </c>
     </row>
@@ -4021,12 +4021,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Sai Kung - Kin Choi</t>
+          <t>Yuen Long - Fu Yan</t>
         </is>
       </c>
     </row>
@@ -4036,12 +4036,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Sai Kung - King Lam</t>
+          <t>Yuen Long - Ha Tsuen</t>
         </is>
       </c>
     </row>
@@ -4051,12 +4051,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Sai Kung - Kwong Ming</t>
+          <t>Yuen Long - Kingswood North</t>
         </is>
       </c>
     </row>
@@ -4066,12 +4066,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Sai Kung - Po Hong</t>
+          <t>Yuen Long - Kingswood South</t>
         </is>
       </c>
     </row>
@@ -4081,12 +4081,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Sai Kung - Po Lam</t>
+          <t>Yuen Long - Ping Shan North</t>
         </is>
       </c>
     </row>
@@ -4096,12 +4096,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Sai Kung - Sheung Tak</t>
+          <t>Yuen Long - Shui Oi</t>
         </is>
       </c>
     </row>
@@ -4111,12 +4111,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Sai Kung - Tak Ming</t>
+          <t>Yuen Long - Shui Wah</t>
         </is>
       </c>
     </row>
@@ -4126,12 +4126,12 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Sai Kung - Tseung Kwan O Centre</t>
+          <t>Yuen Long - Tin Heng</t>
         </is>
       </c>
     </row>
@@ -4141,12 +4141,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Sai Kung - Tsui Lam</t>
+          <t>Yuen Long - Tin Shing</t>
         </is>
       </c>
     </row>
@@ -4156,12 +4156,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Sai Kung - Wan Hang</t>
+          <t>Yuen Long - Tin Yiu</t>
         </is>
       </c>
     </row>
@@ -4171,12 +4171,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Sai Kung - Wan Po</t>
+          <t>Yuen Long - Tsz Yau</t>
         </is>
       </c>
     </row>
@@ -4186,12 +4186,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Tseung Kwan O</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Sai Kung - Yan Ying</t>
+          <t>Yuen Long - Wang Yat</t>
         </is>
       </c>
     </row>
@@ -4201,12 +4201,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Chung Estate</t>
+          <t>Yuen Long - Yat Chak</t>
         </is>
       </c>
     </row>
@@ -4216,12 +4216,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tin Shui Wai</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Kwai Shing West Estate</t>
+          <t>Yuen Long - Yuet Yan</t>
         </is>
       </c>
     </row>
@@ -4231,12 +4231,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Lower Tai Wo Hau</t>
+          <t>Kwun Tong - Kwong Tak</t>
         </is>
       </c>
     </row>
@@ -4246,12 +4246,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Kwai Tsing - On Yam</t>
+          <t>Kwun Tong - Tak Tin</t>
         </is>
       </c>
     </row>
@@ -4261,12 +4261,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Kwai Tsing - Shek Yam</t>
+          <t>Kwun Tong - Yau Tong Sze Shan East</t>
         </is>
       </c>
     </row>
@@ -4276,12 +4276,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Allway</t>
+          <t>Kwun Tong - Yau Tong Sze Shan West</t>
         </is>
       </c>
     </row>
@@ -4291,12 +4291,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Cheung Shek</t>
+          <t>Sai Kung - Fu Yu</t>
         </is>
       </c>
     </row>
@@ -4306,12 +4306,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Clague Garden</t>
+          <t>Sai Kung - Hang Hau East</t>
         </is>
       </c>
     </row>
@@ -4321,12 +4321,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Discovery Park</t>
+          <t>Sai Kung - Hang Hau West</t>
         </is>
       </c>
     </row>
@@ -4336,12 +4336,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Fuk Loi</t>
+          <t>Sai Kung - Hau Tak</t>
         </is>
       </c>
     </row>
@@ -4351,12 +4351,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Hoi Bun</t>
+          <t>Sai Kung - Hong King</t>
         </is>
       </c>
     </row>
@@ -4366,12 +4366,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lai Hing</t>
+          <t>Sai Kung - Kin Choi</t>
         </is>
       </c>
     </row>
@@ -4381,12 +4381,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lai To</t>
+          <t>Sai Kung - King Lam</t>
         </is>
       </c>
     </row>
@@ -4396,12 +4396,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lei Muk Shue East</t>
+          <t>Sai Kung - Kwong Ming</t>
         </is>
       </c>
     </row>
@@ -4411,12 +4411,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Lei Muk Shue West</t>
+          <t>Sai Kung - Po Hong</t>
         </is>
       </c>
     </row>
@@ -4426,12 +4426,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Luk Yeung</t>
+          <t>Sai Kung - Po Lam</t>
         </is>
       </c>
     </row>
@@ -4441,12 +4441,12 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Shek Wai Kok</t>
+          <t>Sai Kung - Sheung Tak</t>
         </is>
       </c>
     </row>
@@ -4456,12 +4456,12 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tak Wah</t>
+          <t>Sai Kung - Tak Ming</t>
         </is>
       </c>
     </row>
@@ -4471,12 +4471,12 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tsuen Wan Centre</t>
+          <t>Sai Kung - Tseung Kwan O Centre</t>
         </is>
       </c>
     </row>
@@ -4486,12 +4486,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tsuen Wan Rural East</t>
+          <t>Sai Kung - Tsui Lam</t>
         </is>
       </c>
     </row>
@@ -4501,12 +4501,12 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tsuen Wan Rural West</t>
+          <t>Sai Kung - Wan Hang</t>
         </is>
       </c>
     </row>
@@ -4516,12 +4516,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Yeung Uk Road</t>
+          <t>Sai Kung - Wan Po</t>
         </is>
       </c>
     </row>
@@ -4531,12 +4531,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
+          <t>Tseung Kwan O</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Tuen Mun - Sam Shing</t>
+          <t>Sai Kung - Yan Ying</t>
         </is>
       </c>
     </row>
@@ -4546,12 +4546,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Tsuen Wan - Tsuen Wan Rural West</t>
+          <t>Kwai Tsing - Kwai Chung Estate</t>
         </is>
       </c>
     </row>
@@ -4561,12 +4561,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Tuen Mun - Butterfly</t>
+          <t>Kwai Tsing - Kwai Shing West Estate</t>
         </is>
       </c>
     </row>
@@ -4576,12 +4576,12 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Tuen Mun - Fu Tai</t>
+          <t>Kwai Tsing - Lower Tai Wo Hau</t>
         </is>
       </c>
     </row>
@@ -4591,12 +4591,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Tuen Mun - Hanford</t>
+          <t>Kwai Tsing - On Yam</t>
         </is>
       </c>
     </row>
@@ -4606,12 +4606,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Tuen Mun - Hing Tsak</t>
+          <t>Kwai Tsing - Shek Yam</t>
         </is>
       </c>
     </row>
@@ -4621,12 +4621,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Tuen Mun - Kin Sang</t>
+          <t>Tsuen Wan - Allway</t>
         </is>
       </c>
     </row>
@@ -4636,12 +4636,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Tuen Mun - King Hing</t>
+          <t>Tsuen Wan - Cheung Shek</t>
         </is>
       </c>
     </row>
@@ -4651,12 +4651,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Tuen Mun - Leung King</t>
+          <t>Tsuen Wan - Clague Garden</t>
         </is>
       </c>
     </row>
@@ -4666,12 +4666,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Tuen Mun - Lok Tsui</t>
+          <t>Tsuen Wan - Discovery Park</t>
         </is>
       </c>
     </row>
@@ -4681,12 +4681,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Tuen Mun - Lung Mun</t>
+          <t>Tsuen Wan - Fuk Loi</t>
         </is>
       </c>
     </row>
@@ -4696,12 +4696,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Tuen Mun - On Ting</t>
+          <t>Tsuen Wan - Hoi Bun</t>
         </is>
       </c>
     </row>
@@ -4711,12 +4711,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Tuen Mun - Po Tin</t>
+          <t>Tsuen Wan - Lai Hing</t>
         </is>
       </c>
     </row>
@@ -4726,12 +4726,12 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Tuen Mun - Prime View</t>
+          <t>Tsuen Wan - Lai To</t>
         </is>
       </c>
     </row>
@@ -4741,12 +4741,12 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Tuen Mun - Sam Shing</t>
+          <t>Tsuen Wan - Lei Muk Shue East</t>
         </is>
       </c>
     </row>
@@ -4756,12 +4756,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Tuen Mun - San Hui</t>
+          <t>Tsuen Wan - Lei Muk Shue West</t>
         </is>
       </c>
     </row>
@@ -4771,12 +4771,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Tuen Mun - San King</t>
+          <t>Tsuen Wan - Luk Yeung</t>
         </is>
       </c>
     </row>
@@ -4786,12 +4786,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Tuen Mun - Shan King</t>
+          <t>Tsuen Wan - Shek Wai Kok</t>
         </is>
       </c>
     </row>
@@ -4801,12 +4801,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Chi</t>
+          <t>Tsuen Wan - Tak Wah</t>
         </is>
       </c>
     </row>
@@ -4816,12 +4816,12 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Hei</t>
+          <t>Tsuen Wan - Tsuen Wan Centre</t>
         </is>
       </c>
     </row>
@@ -4831,12 +4831,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Hong</t>
+          <t>Tsuen Wan - Tsuen Wan Rural East</t>
         </is>
       </c>
     </row>
@@ -4846,12 +4846,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Sun</t>
+          <t>Tsuen Wan - Tsuen Wan Rural West</t>
         </is>
       </c>
     </row>
@@ -4861,12 +4861,12 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Tuen Mun - Siu Tsui</t>
+          <t>Tsuen Wan - Yeung Uk Road</t>
         </is>
       </c>
     </row>
@@ -4876,12 +4876,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Tuen Mun</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tin King</t>
+          <t>Tuen Mun - Sam Shing</t>
         </is>
       </c>
     </row>
@@ -4896,7 +4896,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tsui Hing</t>
+          <t>Tsuen Wan - Tsuen Wan Rural West</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tuen Mun Rural</t>
+          <t>Tuen Mun - Butterfly</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Tuen Mun - Tuen Mun Town Centre</t>
+          <t>Tuen Mun - Fu Tai</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Tuen Mun - Wu King</t>
+          <t>Tuen Mun - Hanford</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Tuen Mun - Yau Oi North</t>
+          <t>Tuen Mun - Hing Tsak</t>
         </is>
       </c>
     </row>
@@ -4971,7 +4971,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Tuen Mun - Yau Oi South</t>
+          <t>Tuen Mun - Kin Sang</t>
         </is>
       </c>
     </row>
@@ -4986,7 +4986,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Tuen Mun - Yuet Wu</t>
+          <t>Tuen Mun - King Hing</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Yuen Long - Ha Tsuen</t>
+          <t>Tuen Mun - Leung King</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Yuen Long - Ping Shan South</t>
+          <t>Tuen Mun - Lok Tsui</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5031,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Yuen Long - Shap Pat Heung South</t>
+          <t>Tuen Mun - Lung Mun</t>
         </is>
       </c>
     </row>
@@ -5041,12 +5041,12 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Yuen Long - Fung Cheung</t>
+          <t>Tuen Mun - On Ting</t>
         </is>
       </c>
     </row>
@@ -5056,12 +5056,12 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Yuen Long - Fung Nin</t>
+          <t>Tuen Mun - Po Tin</t>
         </is>
       </c>
     </row>
@@ -5071,12 +5071,12 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Yuen Long - Nam Ping</t>
+          <t>Tuen Mun - Prime View</t>
         </is>
       </c>
     </row>
@@ -5086,12 +5086,12 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Yuen Long - Pek Long</t>
+          <t>Tuen Mun - Sam Shing</t>
         </is>
       </c>
     </row>
@@ -5101,12 +5101,12 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Yuen Long - Ping Shan North</t>
+          <t>Tuen Mun - San Hui</t>
         </is>
       </c>
     </row>
@@ -5116,12 +5116,12 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Yuen Long - Ping Shan South</t>
+          <t>Tuen Mun - San King</t>
         </is>
       </c>
     </row>
@@ -5131,12 +5131,12 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Yuen Long - San Tin</t>
+          <t>Tuen Mun - Shan King</t>
         </is>
       </c>
     </row>
@@ -5146,12 +5146,12 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Yuen Long - Shap Pat Heung North</t>
+          <t>Tuen Mun - Siu Chi</t>
         </is>
       </c>
     </row>
@@ -5161,12 +5161,12 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Yuen Long - Shap Pat Heung South</t>
+          <t>Tuen Mun - Siu Hei</t>
         </is>
       </c>
     </row>
@@ -5176,12 +5176,12 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Yuen Long</t>
+          <t>Tuen Mun</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Yuen Long - Shui Pin</t>
+          <t>Tuen Mun - Siu Hong</t>
         </is>
       </c>
     </row>
@@ -5191,10 +5191,355 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Siu Sun</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Siu Tsui</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Tin King</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Tsui Hing</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Tuen Mun Rural</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Tuen Mun Town Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Wu King</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Yau Oi North</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Yau Oi South</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Tuen Mun - Yuet Wu</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Yuen Long - Ha Tsuen</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Yuen Long - Ping Shan South</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Tuen Mun</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Yuen Long - Shap Pat Heung South</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
           <t>Yuen Long</t>
         </is>
       </c>
-      <c r="C317" t="inlineStr">
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Yuen Long - Fung Cheung</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Yuen Long - Fung Nin</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Yuen Long - Nam Ping</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Yuen Long - Pek Long</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Yuen Long - Ping Shan North</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Yuen Long - Ping Shan South</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Yuen Long - San Tin</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Yuen Long - Shap Pat Heung North</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Yuen Long - Shap Pat Heung South</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Yuen Long - Shui Pin</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Yuen Long</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
         <is>
           <t>Yuen Long - Tai Kiu</t>
         </is>

</xml_diff>